<commit_message>
FIxed some type errors and other bugs
</commit_message>
<xml_diff>
--- a/tests/excel_test.xlsx
+++ b/tests/excel_test.xlsx
@@ -1,149 +1,59 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25128"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Coding\Python\Packages\easierexcel\tests\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83466659-C4B8-4F2A-85E5-5EF10ABAD778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="228" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="228" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet 2" sheetId="2" r:id="rId2"/>
-    <sheet name="Links" sheetId="3" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet 2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Links" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet 1'!$A$1:$D$1</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Birth Month</t>
-  </si>
-  <si>
-    <t>Birth Year</t>
-  </si>
-  <si>
-    <t>Age</t>
-  </si>
-  <si>
-    <t>Michael</t>
-  </si>
-  <si>
-    <t>April</t>
-  </si>
-  <si>
-    <t>John</t>
-  </si>
-  <si>
-    <t>May</t>
-  </si>
-  <si>
-    <t>Brian</t>
-  </si>
-  <si>
-    <t>June</t>
-  </si>
-  <si>
-    <t>Allison</t>
-  </si>
-  <si>
-    <t>July</t>
-  </si>
-  <si>
-    <t>Daniel</t>
-  </si>
-  <si>
-    <t>August</t>
-  </si>
-  <si>
-    <t>Rob</t>
-  </si>
-  <si>
-    <t>September</t>
-  </si>
-  <si>
-    <t>October</t>
-  </si>
-  <si>
-    <t>Percent</t>
-  </si>
-  <si>
-    <t>Price</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Hours</t>
-  </si>
-  <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>Test 1</t>
-  </si>
-  <si>
-    <t>Website</t>
-  </si>
-  <si>
-    <t>Tony Stark</t>
-  </si>
-  <si>
-    <t>=HYPERLINK(https://www.Stark.com/","Website")"</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dddd\,\ mmmm\ d\,\ yyyy"/>
   </numFmts>
   <fonts count="4">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="16"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="16"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="10"/>
+      <sz val="11"/>
+      <u val="single"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -227,81 +137,140 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="5"/>
   </cellStyleXfs>
   <cellXfs count="21">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment shrinkToFit="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="full_date_format" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="full_date_format" xfId="2"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -567,244 +536,300 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="8.85546875" style="15" customWidth="1"/>
-    <col min="2" max="2" width="30.7109375" style="4" customWidth="1"/>
-    <col min="3" max="3" width="18.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.28515625" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="247" width="9.140625" style="2" customWidth="1"/>
-    <col min="248" max="16384" width="9.140625" style="2"/>
+    <col width="8.85546875" customWidth="1" style="15" min="1" max="1"/>
+    <col width="30.7109375" customWidth="1" style="4" min="2" max="2"/>
+    <col width="18.28515625" bestFit="1" customWidth="1" style="4" min="3" max="3"/>
+    <col width="9.28515625" bestFit="1" customWidth="1" style="5" min="4" max="4"/>
+    <col width="9.140625" customWidth="1" style="2" min="5" max="247"/>
+    <col width="9.140625" customWidth="1" style="2" min="248" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" ht="72" customHeight="1" thickBot="1">
-      <c r="A1" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="9" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" s="13" customFormat="1">
-      <c r="A2" s="14" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="12">
+    <row r="1" ht="72" customFormat="1" customHeight="1" s="1" thickBot="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Birth Month</t>
+        </is>
+      </c>
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>Birth Year</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>Age</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" customFormat="1" s="13">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>Michael</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>April</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="n">
         <v>1991</v>
       </c>
-      <c r="D2" s="8">
+      <c r="D2" s="8" t="n">
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:4" s="13" customFormat="1">
-      <c r="A3" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="12">
+    <row r="3" customFormat="1" s="13">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>John</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="C3" s="12" t="n">
         <v>1990</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="8" t="n">
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:4" s="13" customFormat="1">
-      <c r="A4" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="12">
+    <row r="4" customFormat="1" s="13">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>June</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="n">
         <v>1989</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="8" t="n">
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:4" s="13" customFormat="1">
-      <c r="A5" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="12">
+    <row r="5" customFormat="1" s="13">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>Allison</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>July</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="n">
         <v>1988</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="8" t="n">
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:4" s="13" customFormat="1">
-      <c r="A6" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="12">
+    <row r="6" customFormat="1" s="13">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>Daniel</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>August</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="n">
         <v>1987</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="8" t="n">
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:4" s="13" customFormat="1">
-      <c r="A7" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="12">
+    <row r="7" customFormat="1" s="13">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>Rob</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>September</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="n">
         <v>1986</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="8" t="n">
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="14">
+    <row r="8">
+      <c r="A8" s="14" t="n">
         <v>123</v>
       </c>
-      <c r="B8" s="12" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="12">
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>October</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="n">
         <v>1986</v>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="8" t="n">
         <v>36</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:D1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col width="23.28515625" bestFit="1" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="21.75" customHeight="1">
-      <c r="A1" s="16" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="D1" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="E1" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="F1" s="17" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" s="18">
+    <row r="1" ht="21.75" customHeight="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B1" s="17" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
+      </c>
+      <c r="C1" s="17" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="D1" s="17" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="E1" s="17" t="inlineStr">
+        <is>
+          <t>Hours</t>
+        </is>
+      </c>
+      <c r="F1" s="17" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Test 1</t>
+        </is>
+      </c>
+      <c r="B2" s="18" t="n">
         <v>0.5</v>
       </c>
-      <c r="C2" s="19">
+      <c r="C2" s="19" t="n">
         <v>24.99</v>
       </c>
-      <c r="D2" s="20">
+      <c r="D2" s="20" t="n">
         <v>45345</v>
       </c>
-      <c r="E2" s="18">
+      <c r="E2" s="18" t="n">
         <v>2.5</v>
       </c>
-      <c r="F2" s="18">
+      <c r="F2" s="18" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
-      <c r="A3" s="3"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" s="3"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" s="3"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" s="3"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" s="3"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" s="3"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" s="3"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="A10" s="3"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="A11" s="3"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-    </row>
-    <row r="12" spans="1:6">
-      <c r="A12" s="3"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
+    <row r="3">
+      <c r="A3" s="3" t="n"/>
+      <c r="B3" s="4" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="4" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n"/>
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="4" t="n"/>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n"/>
+      <c r="B8" s="4" t="n"/>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n"/>
+      <c r="B9" s="4" t="n"/>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n"/>
+      <c r="B10" s="4" t="n"/>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n"/>
+      <c r="B11" s="4" t="n"/>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n"/>
+      <c r="B12" s="4" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:A12">
@@ -825,28 +850,40 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="47.42578125" bestFit="1" customWidth="1"/>
+    <col width="13.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="47.42578125" bestFit="1" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="21.75" customHeight="1" thickBot="1">
-      <c r="A1" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" s="11" t="s">
-        <v>25</v>
+    <row r="1" ht="21.75" customHeight="1" thickBot="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Tony Stark</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>=HYPERLINK(https://www.Stark.com/","Website")"</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>